<commit_message>
Update Excel datasets and forecast outputs
Replace three Excel files with updated versions: UTR221_zeros_preenchidos.xlsx (zeros filled), inferencia_1h_nivel221.xlsx (1-hour level inference), and real_vs_previsto_ultimas_12h.xlsx (real vs predicted — last 12h). These are binary data/analysis updates containing refreshed data and revised forecasts.
</commit_message>
<xml_diff>
--- a/inferencia_1h_nivel221.xlsx
+++ b/inferencia_1h_nivel221.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,29 +433,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Previsto (m)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Real (m)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Erro (m)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46067.45833333334</v>
       </c>
       <c r="B2" t="n">
@@ -457,7 +469,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46067.46875</v>
       </c>
       <c r="B3" t="n">
@@ -471,7 +483,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46067.47916666666</v>
       </c>
       <c r="B4" t="n">
@@ -485,7 +497,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46067.48958333334</v>
       </c>
       <c r="B5" t="n">

</xml_diff>